<commit_message>
Add Phase 1 household demand and supply-demand equilibrium
</commit_message>
<xml_diff>
--- a/data/Simulation_Settings.xlsx
+++ b/data/Simulation_Settings.xlsx
@@ -2,12 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5176d79aca9c402d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="R7c1c474819dc462a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="Ra36f43d63183422b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="R65ed84bf11b34ccb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="Rbe039ad6dfaf4895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="Rc7036f26a5a64f36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R44f8e0b542294018"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="R297463f082664c68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="Rf7e9ee5d297841de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="R7737e2fe66494ba7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="R4e5b066fddb64cf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="R99481a939ff0406c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption_Baskets" sheetId="7" r:id="R7ec60cf3df134d7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase1_Model" sheetId="8" r:id="Ra26bbcd880c14a4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,12 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="0.00%"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
     <x:numFmt numFmtId="203" formatCode="$#,##0"/>
     <x:numFmt numFmtId="204" formatCode="$#,##0.00"/>
+    <x:numFmt numFmtId="205" formatCode="0.00"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -53,7 +56,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,6 +88,21 @@
         <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -93,7 +111,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="76">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -178,6 +196,46 @@
     <x:xf numFmtId="204" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -189,7 +247,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -200,7 +258,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -211,7 +269,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -222,7 +280,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -602,6 +660,14 @@
       <x:c r="E1" s="10"/>
       <x:c r="F1" s="10"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11"/>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+    </x:row>
     <x:row r="3">
       <x:c r="A3" s="20" t="str">
         <x:v>Key</x:v>
@@ -623,183 +689,343 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="str">
+      <x:c r="A4" s="11" t="str">
         <x:v>target_gini</x:v>
       </x:c>
-      <x:c r="B4" t="str">
+      <x:c r="B4" s="11" t="str">
         <x:v>Gini coefficient</x:v>
       </x:c>
-      <x:c r="C4" s="30" t="n">
+      <x:c r="C4" s="61" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="D4" t="str">
+      <x:c r="D4" s="11" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="E4" t="str">
+      <x:c r="E4" s="11" t="str">
         <x:v>Used</x:v>
       </x:c>
-      <x:c r="F4" t="str">
+      <x:c r="F4" s="11" t="str">
         <x:v>Target Gini for household gross income.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
+      <x:c r="A5" s="11" t="str">
         <x:v>tax_rate</x:v>
       </x:c>
-      <x:c r="B5" t="str">
+      <x:c r="B5" s="11" t="str">
         <x:v>Taxes</x:v>
       </x:c>
-      <x:c r="C5" s="30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D5" t="str">
+      <x:c r="C5" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
         <x:v>% of gross income</x:v>
       </x:c>
-      <x:c r="E5" t="str">
+      <x:c r="E5" s="11" t="str">
         <x:v>Used</x:v>
       </x:c>
-      <x:c r="F5" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>Flat household income-tax placeholder.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
+      <x:c r="A6" s="11" t="str">
         <x:v>interest_rate</x:v>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c r="B6" s="11" t="str">
         <x:v>Interest rate</x:v>
       </x:c>
-      <x:c r="C6" s="30" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D6" t="str">
+      <x:c r="C6" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
         <x:v>% annual</x:v>
       </x:c>
-      <x:c r="E6" t="str">
+      <x:c r="E6" s="11" t="str">
         <x:v>Stored</x:v>
       </x:c>
-      <x:c r="F6" t="str">
+      <x:c r="F6" s="11" t="str">
         <x:v>For future saving, credit, and investment logic.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="str">
+      <x:c r="A7" s="11" t="str">
         <x:v>annual_inflation</x:v>
       </x:c>
-      <x:c r="B7" t="str">
+      <x:c r="B7" s="11" t="str">
         <x:v>Inflation</x:v>
       </x:c>
-      <x:c r="C7" s="30" t="n">
+      <x:c r="C7" s="61" t="n">
         <x:v>0.02</x:v>
       </x:c>
-      <x:c r="D7" t="str">
+      <x:c r="D7" s="11" t="str">
         <x:v>% annual</x:v>
       </x:c>
-      <x:c r="E7" t="str">
+      <x:c r="E7" s="11" t="str">
         <x:v>Used</x:v>
       </x:c>
-      <x:c r="F7" t="str">
+      <x:c r="F7" s="11" t="str">
         <x:v>Median annual inflation target.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="str">
+      <x:c r="A8" s="11" t="str">
         <x:v>num_households</x:v>
       </x:c>
-      <x:c r="B8" t="str">
+      <x:c r="B8" s="11" t="str">
         <x:v>Number of consumers / households</x:v>
       </x:c>
-      <x:c r="C8" s="32" t="n">
+      <x:c r="C8" s="62" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="D8" t="str">
+      <x:c r="D8" s="11" t="str">
         <x:v>households</x:v>
       </x:c>
-      <x:c r="E8" t="str">
+      <x:c r="E8" s="11" t="str">
         <x:v>Used</x:v>
       </x:c>
-      <x:c r="F8" t="str">
+      <x:c r="F8" s="11" t="str">
         <x:v>Number of household agents.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="str">
+      <x:c r="A9" s="11" t="str">
         <x:v>num_companies</x:v>
       </x:c>
-      <x:c r="B9" t="str">
+      <x:c r="B9" s="11" t="str">
         <x:v>Number of companies</x:v>
       </x:c>
-      <x:c r="C9" s="32" t="n">
+      <x:c r="C9" s="62" t="n">
         <x:v>1000</x:v>
       </x:c>
-      <x:c r="D9" t="str">
+      <x:c r="D9" s="11" t="str">
         <x:v>companies</x:v>
       </x:c>
-      <x:c r="E9" t="str">
+      <x:c r="E9" s="11" t="str">
         <x:v>Used</x:v>
       </x:c>
-      <x:c r="F9" t="str">
+      <x:c r="F9" s="11" t="str">
         <x:v>Number of company agents.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="str">
+      <x:c r="A10" s="11" t="str">
         <x:v>simulation_years</x:v>
       </x:c>
-      <x:c r="B10" t="str">
+      <x:c r="B10" s="11" t="str">
         <x:v>Years of simulation</x:v>
       </x:c>
-      <x:c r="C10" s="32" t="n">
+      <x:c r="C10" s="62" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D10" t="str">
+      <x:c r="D10" s="11" t="str">
         <x:v>years</x:v>
       </x:c>
-      <x:c r="E10" t="str">
+      <x:c r="E10" s="11" t="str">
         <x:v>Used</x:v>
       </x:c>
-      <x:c r="F10" t="str">
+      <x:c r="F10" s="11" t="str">
         <x:v>The model evaluates equilibrium every month.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="str">
+      <x:c r="A11" s="11" t="str">
         <x:v>random_seed</x:v>
       </x:c>
-      <x:c r="B11" t="str">
+      <x:c r="B11" s="11" t="str">
         <x:v>Random seed</x:v>
       </x:c>
-      <x:c r="C11" s="32" t="n">
+      <x:c r="C11" s="62" t="n">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="D11" t="str">
+      <x:c r="D11" s="11" t="str">
         <x:v>integer</x:v>
       </x:c>
-      <x:c r="E11" t="str">
+      <x:c r="E11" s="11" t="str">
         <x:v>Used</x:v>
       </x:c>
-      <x:c r="F11" t="str">
+      <x:c r="F11" s="11" t="str">
         <x:v>Keep fixed for reproducibility; change for another starting economy.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="str">
+      <x:c r="A12" s="11" t="str">
         <x:v>monthly_price_noise_std</x:v>
       </x:c>
-      <x:c r="B12" t="str">
+      <x:c r="B12" s="11" t="str">
         <x:v>Monthly price dispersion</x:v>
       </x:c>
-      <x:c r="C12" s="30" t="n">
+      <x:c r="C12" s="61" t="n">
         <x:v>0.0025</x:v>
       </x:c>
-      <x:c r="D12" t="str">
+      <x:c r="D12" s="11" t="str">
         <x:v>decimal</x:v>
       </x:c>
-      <x:c r="E12" t="str">
+      <x:c r="E12" s="11" t="str">
         <x:v>Used</x:v>
       </x:c>
-      <x:c r="F12" t="str">
+      <x:c r="F12" s="11" t="str">
         <x:v>Random spread around inflation/12. Allows occasional price decreases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="11" t="str">
+        <x:v>demographic_growth</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>Annual household growth</x:v>
+      </x:c>
+      <x:c r="C13" s="63" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="str">
+        <x:v>% annual</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F13" s="11" t="str">
+        <x:v>Applied once per year. Default 1% adds households while preserving class proportions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="11" t="str">
+        <x:v>company_growth_sensitivity</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="str">
+        <x:v>Company growth sensitivity</x:v>
+      </x:c>
+      <x:c r="C14" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="str">
+        <x:v>multiplier</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F14" s="11" t="str">
+        <x:v>New-company rate = positive prior-year real GDP growth × this sensitivity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="11" t="str">
+        <x:v>allow_company_exits</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="str">
+        <x:v>Allow company exits in recession</x:v>
+      </x:c>
+      <x:c r="C15" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="str">
+        <x:v>0/1</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F15" s="11" t="str">
+        <x:v>0 = no automatic exits; 1 = negative prior-year real GDP growth can reduce company count.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="11" t="str">
+        <x:v>price_adjustment_speed</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="str">
+        <x:v>Supply-demand price adjustment</x:v>
+      </x:c>
+      <x:c r="C16" s="64" t="n">
+        <x:v>0.12</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="str">
+        <x:v>coefficient</x:v>
+      </x:c>
+      <x:c r="E16" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F16" s="11" t="str">
+        <x:v>Higher value makes shortages/surpluses change prices faster.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="11" t="str">
+        <x:v>production_adjustment_speed</x:v>
+      </x:c>
+      <x:c r="B17" s="11" t="str">
+        <x:v>Production adjustment speed</x:v>
+      </x:c>
+      <x:c r="C17" s="64" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="str">
+        <x:v>coefficient</x:v>
+      </x:c>
+      <x:c r="E17" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F17" s="11" t="str">
+        <x:v>How strongly next month's production responds to current demand/supply imbalance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="11" t="str">
+        <x:v>max_monthly_price_change</x:v>
+      </x:c>
+      <x:c r="B18" s="11" t="str">
+        <x:v>Max monthly price movement</x:v>
+      </x:c>
+      <x:c r="C18" s="63" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="E18" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F18" s="11" t="str">
+        <x:v>Absolute cap on an individual product's monthly price change.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="11" t="str">
+        <x:v>max_monthly_production_change</x:v>
+      </x:c>
+      <x:c r="B19" s="11" t="str">
+        <x:v>Max monthly production movement</x:v>
+      </x:c>
+      <x:c r="C19" s="63" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="D19" s="11" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="E19" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F19" s="11" t="str">
+        <x:v>Absolute cap on an individual product's monthly production change.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="11" t="str">
+        <x:v>initial_inventory_months</x:v>
+      </x:c>
+      <x:c r="B20" s="11" t="str">
+        <x:v>Initial inventory</x:v>
+      </x:c>
+      <x:c r="C20" s="75" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D20" s="11" t="str">
+        <x:v>months of P0 output</x:v>
+      </x:c>
+      <x:c r="E20" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F20" s="11" t="str">
+        <x:v>Starts at zero so Period 0 is an exact demand=supply equilibrium. Inventory then forms from unsold output.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5432,4 +5658,657 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="33" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="54" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="73" t="str">
+        <x:v>Household Consumption Basket Preference Multipliers</x:v>
+      </x:c>
+      <x:c r="B1" s="73"/>
+      <x:c r="C1" s="73"/>
+      <x:c r="D1" s="73"/>
+      <x:c r="E1" s="73"/>
+      <x:c r="F1" s="73"/>
+      <x:c r="G1" s="73"/>
+      <x:c r="H1" s="73"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11" t="str">
+        <x:v>Yellow cells are relative preferences, not percentages. 1.00 = neutral. The simulation calibrates these preferences so Period-0 class budgets and product sales both reconcile exactly.</x:v>
+      </x:c>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+      <x:c r="G2" s="11"/>
+      <x:c r="H2" s="11"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="11"/>
+      <x:c r="C3" s="11"/>
+      <x:c r="D3" s="11"/>
+      <x:c r="E3" s="11"/>
+      <x:c r="F3" s="11"/>
+      <x:c r="G3" s="11"/>
+      <x:c r="H3" s="11"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="72" t="str">
+        <x:v>Division</x:v>
+      </x:c>
+      <x:c r="B4" s="72" t="str">
+        <x:v>COICOP Division</x:v>
+      </x:c>
+      <x:c r="C4" s="72" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="D4" s="72" t="str">
+        <x:v>Middle</x:v>
+      </x:c>
+      <x:c r="E4" s="72" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="F4" s="72" t="str">
+        <x:v>Top 1%</x:v>
+      </x:c>
+      <x:c r="G4" s="72" t="str">
+        <x:v>Top 0.1%</x:v>
+      </x:c>
+      <x:c r="H4" s="72" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="str">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Food &amp; non-alcoholic beverages</x:v>
+      </x:c>
+      <x:c r="C5" s="64" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
+      <x:c r="D5" s="64" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="E5" s="64" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="F5" s="64" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="G5" s="64" t="n">
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="H5" s="11" t="str">
+        <x:v>Lower-income households place more relative weight here.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="str">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Alcohol &amp; tobacco</x:v>
+      </x:c>
+      <x:c r="C6" s="64" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="D6" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" s="64" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="F6" s="64" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="G6" s="64" t="n">
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="H6" s="11" t="str">
+        <x:v>Editable behavioral assumption.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="str">
+        <x:v>03</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>Clothing &amp; footwear</x:v>
+      </x:c>
+      <x:c r="C7" s="64" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="D7" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="64" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="F7" s="64" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="G7" s="64" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="H7" s="11" t="str">
+        <x:v>Higher-income households place more relative weight here.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="str">
+        <x:v>04</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>Housing &amp; utilities</x:v>
+      </x:c>
+      <x:c r="C8" s="64" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="D8" s="64" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="E8" s="64" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="F8" s="64" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="G8" s="64" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="H8" s="11" t="str">
+        <x:v>Large relative burden for lower-income households.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="str">
+        <x:v>05</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Furnishings &amp; maintenance</x:v>
+      </x:c>
+      <x:c r="C9" s="64" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="D9" s="64" t="n">
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="E9" s="64" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="F9" s="64" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
+      <x:c r="G9" s="64" t="n">
+        <x:v>1.45</x:v>
+      </x:c>
+      <x:c r="H9" s="11" t="str">
+        <x:v>Higher discretionary weight at higher incomes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="str">
+        <x:v>06</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>Health</x:v>
+      </x:c>
+      <x:c r="C10" s="64" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="D10" s="64" t="n">
+        <x:v>1.05</x:v>
+      </x:c>
+      <x:c r="E10" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F10" s="64" t="n">
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="G10" s="64" t="n">
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="H10" s="11" t="str">
+        <x:v>Slightly higher relative burden at lower incomes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="11" t="str">
+        <x:v>07</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
+        <x:v>Transport</x:v>
+      </x:c>
+      <x:c r="C11" s="64" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="D11" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E11" s="64" t="n">
+        <x:v>1.1</x:v>
+      </x:c>
+      <x:c r="F11" s="64" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="G11" s="64" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
+      <x:c r="H11" s="11" t="str">
+        <x:v>Higher-income households can spend more on higher-value transport.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="11" t="str">
+        <x:v>08</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="str">
+        <x:v>Communication</x:v>
+      </x:c>
+      <x:c r="C12" s="64" t="n">
+        <x:v>1.05</x:v>
+      </x:c>
+      <x:c r="D12" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="64" t="n">
+        <x:v>0.95</x:v>
+      </x:c>
+      <x:c r="F12" s="64" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="G12" s="64" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="H12" s="11" t="str">
+        <x:v>Relatively essential across classes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="11" t="str">
+        <x:v>09</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>Recreation</x:v>
+      </x:c>
+      <x:c r="C13" s="64" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="D13" s="64" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="E13" s="64" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="F13" s="64" t="n">
+        <x:v>1.55</x:v>
+      </x:c>
+      <x:c r="G13" s="64" t="n">
+        <x:v>1.75</x:v>
+      </x:c>
+      <x:c r="H13" s="11" t="str">
+        <x:v>Strong discretionary-income effect.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="11" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="str">
+        <x:v>Education</x:v>
+      </x:c>
+      <x:c r="C14" s="64" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="D14" s="64" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="64" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="F14" s="64" t="n">
+        <x:v>1.35</x:v>
+      </x:c>
+      <x:c r="G14" s="64" t="n">
+        <x:v>1.45</x:v>
+      </x:c>
+      <x:c r="H14" s="11" t="str">
+        <x:v>Higher-income preference multiplier.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="11" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="str">
+        <x:v>Restaurants &amp; hotels</x:v>
+      </x:c>
+      <x:c r="C15" s="64" t="n">
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="D15" s="64" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="E15" s="64" t="n">
+        <x:v>1.25</x:v>
+      </x:c>
+      <x:c r="F15" s="64" t="n">
+        <x:v>1.65</x:v>
+      </x:c>
+      <x:c r="G15" s="64" t="n">
+        <x:v>1.9</x:v>
+      </x:c>
+      <x:c r="H15" s="11" t="str">
+        <x:v>Strong discretionary-income effect.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="11" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="str">
+        <x:v>Financial, insurance &amp; services</x:v>
+      </x:c>
+      <x:c r="C16" s="64" t="n">
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="D16" s="64" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="E16" s="64" t="n">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="F16" s="64" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="G16" s="64" t="n">
+        <x:v>2.2</x:v>
+      </x:c>
+      <x:c r="H16" s="11" t="str">
+        <x:v>Higher use of financial/professional services at higher incomes.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="73" t="str">
+        <x:v>Phase 1 — Monthly Supply/Demand Mechanics</x:v>
+      </x:c>
+      <x:c r="B1" s="73"/>
+      <x:c r="C1" s="73"/>
+      <x:c r="D1" s="73"/>
+      <x:c r="E1" s="73"/>
+      <x:c r="F1" s="73"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11"/>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="72" t="str">
+        <x:v>Step</x:v>
+      </x:c>
+      <x:c r="B3" s="72" t="str">
+        <x:v>Mechanism</x:v>
+      </x:c>
+      <x:c r="C3" s="72" t="str">
+        <x:v>Core idea</x:v>
+      </x:c>
+      <x:c r="D3" s="72" t="str">
+        <x:v>Frequency</x:v>
+      </x:c>
+      <x:c r="E3" s="72" t="str">
+        <x:v>Editable input</x:v>
+      </x:c>
+      <x:c r="F3" s="72" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>Household population</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>Households grow by demographic rate.</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>Annual</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>demographic_growth</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
+        <x:v>Class proportions are preserved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Household budgets</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
+        <x:v>Class consumption budgets grow with population and the prior CPI level.</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>tax_rate</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
+        <x:v>Real per-household baseline income is held constant in Phase 1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Demand basket</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="str">
+        <x:v>Class/product baseline spending is calibrated with basket preference multipliers.</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>P0 + monthly</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>Consumption_Baskets</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>P0 planned spending equals product revenue exactly.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>Elastic demand</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="str">
+        <x:v>Quantity demand responds to each product's price using its 0–1 elasticity.</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>Elasticity_Abs</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="str">
+        <x:v>Class budgets are re-scaled so planned spending stays within budget.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>Inventory &amp; sales</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="str">
+        <x:v>Sales = min(demand, production + beginning inventory).</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
+        <x:v>initial_inventory_months</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
+        <x:v>Unmet demand becomes shortage; unsold supply becomes inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Price response</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="str">
+        <x:v>Background inflation + supply/demand imbalance changes next month's price.</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="str">
+        <x:v>price_adjustment_speed</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="str">
+        <x:v>Price movement is capped.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>Production response</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="str">
+        <x:v>Next month's output responds gradually to demand relative to production.</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>production_adjustment_speed</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:v>Competitive markets react faster; monopoly reacts slower.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
+        <x:v>Company entry</x:v>
+      </x:c>
+      <x:c r="C11" s="11" t="str">
+        <x:v>Positive prior-year real GDP growth creates new companies.</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="str">
+        <x:v>Annual</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="str">
+        <x:v>company_growth_sensitivity</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="str">
+        <x:v>Default sensitivity 1.0 means 3% growth ≈ 3% more firms.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="str">
+        <x:v>Company exit</x:v>
+      </x:c>
+      <x:c r="C12" s="11" t="str">
+        <x:v>Optional recession-driven exits.</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="str">
+        <x:v>Annual</x:v>
+      </x:c>
+      <x:c r="E12" s="11" t="str">
+        <x:v>allow_company_exits</x:v>
+      </x:c>
+      <x:c r="F12" s="11" t="str">
+        <x:v>Disabled by default.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>Macro reporting</x:v>
+      </x:c>
+      <x:c r="C13" s="11" t="str">
+        <x:v>Nominal/real GDP, inflation, shortages, sales, inventory, households and firms.</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="str">
+        <x:v>Monthly + annual</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F13" s="11" t="str">
+        <x:v>Real GDP uses P0 prices.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add intelligent company entry and exit
</commit_message>
<xml_diff>
--- a/data/Simulation_Settings.xlsx
+++ b/data/Simulation_Settings.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R44f8e0b542294018"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="R297463f082664c68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="Rf7e9ee5d297841de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="R7737e2fe66494ba7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="R4e5b066fddb64cf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="R99481a939ff0406c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption_Baskets" sheetId="7" r:id="R7ec60cf3df134d7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase1_Model" sheetId="8" r:id="Ra26bbcd880c14a4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6098a022972544f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="Rb7d2f210aa864172"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="Ra912e2372ed54e2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="R3da449fd49ff47f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="R1a72a7348c0d439a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="Rb902dfc58da54377"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption_Baskets" sheetId="7" r:id="R480e22f7dbf54fc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase1_Model" sheetId="8" r:id="R5bcc1df5933243f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firm_Entry_Exit" sheetId="9" r:id="Reb8ec471b592479b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -56,7 +57,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -103,6 +104,21 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -111,7 +127,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="76">
+  <x:cellXfs count="90">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -234,6 +250,32 @@
     </x:xf>
     <x:xf numFmtId="205" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="205" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -875,7 +917,7 @@
       <x:c r="B13" s="11" t="str">
         <x:v>Annual household growth</x:v>
       </x:c>
-      <x:c r="C13" s="63" t="n">
+      <x:c r="C13" s="61" t="n">
         <x:v>0.01</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
@@ -895,7 +937,7 @@
       <x:c r="B14" s="11" t="str">
         <x:v>Company growth sensitivity</x:v>
       </x:c>
-      <x:c r="C14" s="64" t="n">
+      <x:c r="C14" s="75" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
@@ -915,7 +957,7 @@
       <x:c r="B15" s="11" t="str">
         <x:v>Allow company exits in recession</x:v>
       </x:c>
-      <x:c r="C15" s="64" t="n">
+      <x:c r="C15" s="75" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
@@ -935,7 +977,7 @@
       <x:c r="B16" s="11" t="str">
         <x:v>Supply-demand price adjustment</x:v>
       </x:c>
-      <x:c r="C16" s="64" t="n">
+      <x:c r="C16" s="75" t="n">
         <x:v>0.12</x:v>
       </x:c>
       <x:c r="D16" s="11" t="str">
@@ -955,7 +997,7 @@
       <x:c r="B17" s="11" t="str">
         <x:v>Production adjustment speed</x:v>
       </x:c>
-      <x:c r="C17" s="64" t="n">
+      <x:c r="C17" s="75" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="D17" s="11" t="str">
@@ -975,7 +1017,7 @@
       <x:c r="B18" s="11" t="str">
         <x:v>Max monthly price movement</x:v>
       </x:c>
-      <x:c r="C18" s="63" t="n">
+      <x:c r="C18" s="61" t="n">
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
@@ -995,7 +1037,7 @@
       <x:c r="B19" s="11" t="str">
         <x:v>Max monthly production movement</x:v>
       </x:c>
-      <x:c r="C19" s="63" t="n">
+      <x:c r="C19" s="61" t="n">
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="D19" s="11" t="str">
@@ -1026,6 +1068,246 @@
       </x:c>
       <x:c r="F20" s="11" t="str">
         <x:v>Starts at zero so Period 0 is an exact demand=supply equilibrium. Inventory then forms from unsold output.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="11" t="str">
+        <x:v>entry_shortage_weight</x:v>
+      </x:c>
+      <x:c r="B21" s="11" t="str">
+        <x:v>Entry: shortage weight</x:v>
+      </x:c>
+      <x:c r="C21" s="80" t="n">
+        <x:v>0.45</x:v>
+      </x:c>
+      <x:c r="D21" s="11" t="str">
+        <x:v>weight</x:v>
+      </x:c>
+      <x:c r="E21" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F21" s="11" t="str">
+        <x:v>Share of the entry score driven by persistent unmet demand.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="11" t="str">
+        <x:v>entry_demand_growth_weight</x:v>
+      </x:c>
+      <x:c r="B22" s="11" t="str">
+        <x:v>Entry: demand growth weight</x:v>
+      </x:c>
+      <x:c r="C22" s="80" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="D22" s="11" t="str">
+        <x:v>weight</x:v>
+      </x:c>
+      <x:c r="E22" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F22" s="11" t="str">
+        <x:v>Share of the entry score driven by prior-year product demand growth.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="11" t="str">
+        <x:v>entry_margin_weight</x:v>
+      </x:c>
+      <x:c r="B23" s="11" t="str">
+        <x:v>Entry: profit margin weight</x:v>
+      </x:c>
+      <x:c r="C23" s="80" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="D23" s="11" t="str">
+        <x:v>weight</x:v>
+      </x:c>
+      <x:c r="E23" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F23" s="11" t="str">
+        <x:v>Share of the entry score driven by the product-market operating margin proxy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="11" t="str">
+        <x:v>exit_surplus_weight</x:v>
+      </x:c>
+      <x:c r="B24" s="11" t="str">
+        <x:v>Exit: surplus weight</x:v>
+      </x:c>
+      <x:c r="C24" s="80" t="n">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="D24" s="11" t="str">
+        <x:v>weight</x:v>
+      </x:c>
+      <x:c r="E24" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F24" s="11" t="str">
+        <x:v>Share of the exit score driven by excess ending inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="11" t="str">
+        <x:v>exit_demand_decline_weight</x:v>
+      </x:c>
+      <x:c r="B25" s="11" t="str">
+        <x:v>Exit: demand decline weight</x:v>
+      </x:c>
+      <x:c r="C25" s="80" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="D25" s="11" t="str">
+        <x:v>weight</x:v>
+      </x:c>
+      <x:c r="E25" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F25" s="11" t="str">
+        <x:v>Share of the exit score driven by falling product demand.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="11" t="str">
+        <x:v>exit_loss_weight</x:v>
+      </x:c>
+      <x:c r="B26" s="11" t="str">
+        <x:v>Exit: loss weight</x:v>
+      </x:c>
+      <x:c r="C26" s="80" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="D26" s="11" t="str">
+        <x:v>weight</x:v>
+      </x:c>
+      <x:c r="E26" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F26" s="11" t="str">
+        <x:v>Share of the exit score driven by negative operating margin.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="11" t="str">
+        <x:v>max_entries_per_product</x:v>
+      </x:c>
+      <x:c r="B27" s="11" t="str">
+        <x:v>Max entrants / product / year</x:v>
+      </x:c>
+      <x:c r="C27" s="81" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D27" s="11" t="str">
+        <x:v>firms</x:v>
+      </x:c>
+      <x:c r="E27" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F27" s="11" t="str">
+        <x:v>Prevents all new companies from entering one attractive product market.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="11" t="str">
+        <x:v>max_exits_per_product</x:v>
+      </x:c>
+      <x:c r="B28" s="11" t="str">
+        <x:v>Max exits / product / year</x:v>
+      </x:c>
+      <x:c r="C28" s="81" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D28" s="11" t="str">
+        <x:v>firms</x:v>
+      </x:c>
+      <x:c r="E28" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F28" s="11" t="str">
+        <x:v>Maximum annual exits from a single product; a market never falls below one firm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="11" t="str">
+        <x:v>entry_capacity_share</x:v>
+      </x:c>
+      <x:c r="B29" s="11" t="str">
+        <x:v>Entrant capacity share</x:v>
+      </x:c>
+      <x:c r="C29" s="75" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="D29" s="11" t="str">
+        <x:v>share of avg incumbent</x:v>
+      </x:c>
+      <x:c r="E29" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F29" s="11" t="str">
+        <x:v>One entrant initially adds 15% of average incumbent production capacity. This keeps entry gradual because monthly production adjustment already responds to demand.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="11" t="str">
+        <x:v>exit_capacity_share</x:v>
+      </x:c>
+      <x:c r="B30" s="11" t="str">
+        <x:v>Exit capacity share</x:v>
+      </x:c>
+      <x:c r="C30" s="80" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D30" s="11" t="str">
+        <x:v>share of avg incumbent</x:v>
+      </x:c>
+      <x:c r="E30" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F30" s="11" t="str">
+        <x:v>One exiting firm removes this fraction of average incumbent production capacity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="11" t="str">
+        <x:v>min_entry_score</x:v>
+      </x:c>
+      <x:c r="B31" s="11" t="str">
+        <x:v>Minimum entry score</x:v>
+      </x:c>
+      <x:c r="C31" s="80" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="D31" s="11" t="str">
+        <x:v>0–1 score</x:v>
+      </x:c>
+      <x:c r="E31" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F31" s="11" t="str">
+        <x:v>Markets below this score normally do not receive entrants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="11" t="str">
+        <x:v>min_exit_score</x:v>
+      </x:c>
+      <x:c r="B32" s="11" t="str">
+        <x:v>Minimum exit score</x:v>
+      </x:c>
+      <x:c r="C32" s="80" t="n">
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="D32" s="11" t="str">
+        <x:v>0–1 score</x:v>
+      </x:c>
+      <x:c r="E32" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F32" s="11" t="str">
+        <x:v>A weak market must reach this score before recession-driven exits are allocated.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6311,4 +6593,202 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="43" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="54" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="88" t="str">
+        <x:v>Intelligent Company Entry / Exit — Phase 1.1</x:v>
+      </x:c>
+      <x:c r="B1" s="88"/>
+      <x:c r="C1" s="88"/>
+      <x:c r="D1" s="88"/>
+      <x:c r="E1" s="88"/>
+      <x:c r="F1" s="88"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11"/>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="87" t="str">
+        <x:v>Step</x:v>
+      </x:c>
+      <x:c r="B3" s="87" t="str">
+        <x:v>Decision</x:v>
+      </x:c>
+      <x:c r="C3" s="87" t="str">
+        <x:v>Signals</x:v>
+      </x:c>
+      <x:c r="D3" s="87" t="str">
+        <x:v>Effect</x:v>
+      </x:c>
+      <x:c r="E3" s="87" t="str">
+        <x:v>Timing</x:v>
+      </x:c>
+      <x:c r="F3" s="87" t="str">
+        <x:v>Important rule</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>How many firms enter?</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>Prior-year real GDP growth × company growth sensitivity</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>Sets the economy-wide entrant count.</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>Start of each year</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
+        <x:v>Positive real growth creates entrants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Where do entrants go?</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
+        <x:v>Shortage + demand growth + profit margin</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>Higher-score product markets receive more new firms.</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>Start of each year</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
+        <x:v>Allocation is weighted, not random.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Capacity effect</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="str">
+        <x:v>Entrants per product / incumbent firms</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>Raises the selected product's production capacity.</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>Immediately on entry</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>Default entrant adds 15% of average incumbent capacity; monthly production adjustment handles the rest.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>Market structure</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="str">
+        <x:v>Active firms per product</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
+        <x:v>1=Monopoly; 2–4=Oligopoly; 5+=Competitive.</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>After entry/exit</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="str">
+        <x:v>Market structure can now evolve.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>How many firms exit?</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="str">
+        <x:v>Negative real GDP growth × company sensitivity</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
+        <x:v>Sets potential exits only when allow_company_exits=1.</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
+        <x:v>Start of each year</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
+        <x:v>Exits are disabled by default.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Where do exits occur?</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="str">
+        <x:v>Surplus inventory + falling demand + losses</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
+        <x:v>Weak markets lose firms first.</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="str">
+        <x:v>Start of each year</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="str">
+        <x:v>No product can fall below one producer.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>Diagnostics</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="str">
+        <x:v>Entry score, exit score, firm count, market transition</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>Saved to market_events.csv / output workbook.</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>Every annual event</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:v>Product-monthly output records current firm count.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add monthly product innovation
</commit_message>
<xml_diff>
--- a/data/Simulation_Settings.xlsx
+++ b/data/Simulation_Settings.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6098a022972544f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="Rb7d2f210aa864172"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="Ra912e2372ed54e2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="R3da449fd49ff47f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="R1a72a7348c0d439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="Rb902dfc58da54377"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption_Baskets" sheetId="7" r:id="R480e22f7dbf54fc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase1_Model" sheetId="8" r:id="R5bcc1df5933243f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firm_Entry_Exit" sheetId="9" r:id="Reb8ec471b592479b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf8924302aa5743f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="R253b06d823cd4fa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="Rd4cff3d5aa8f4835"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="R62d1a7f3576d4730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="R29d7d3d2066d4907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="R883ffc0e2b6245e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption_Baskets" sheetId="7" r:id="R15f7eba23f944892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase1_Model" sheetId="8" r:id="R4d4c5d067ddb4f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firm_Entry_Exit" sheetId="9" r:id="R763e1afaebae4cdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Innovation" sheetId="10" r:id="Rbae576de4ac14fcf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +58,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -119,6 +120,21 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -127,7 +143,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="90">
+  <x:cellXfs count="107">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -276,6 +292,37 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -680,6 +727,243 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="50" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="104" t="str">
+        <x:v>Monthly Product Innovation / New Product Variants — Phase 1.2</x:v>
+      </x:c>
+      <x:c r="B1" s="104"/>
+      <x:c r="C1" s="104"/>
+      <x:c r="D1" s="104"/>
+      <x:c r="E1" s="104"/>
+      <x:c r="F1" s="104"/>
+      <x:c r="G1" s="104"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11"/>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+      <x:c r="G2" s="11"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="103" t="str">
+        <x:v>Step</x:v>
+      </x:c>
+      <x:c r="B3" s="103" t="str">
+        <x:v>Mechanism</x:v>
+      </x:c>
+      <x:c r="C3" s="103" t="str">
+        <x:v>Default</x:v>
+      </x:c>
+      <x:c r="D3" s="103" t="str">
+        <x:v>Example</x:v>
+      </x:c>
+      <x:c r="E3" s="103" t="str">
+        <x:v>Demand effect</x:v>
+      </x:c>
+      <x:c r="F3" s="103" t="str">
+        <x:v>Production effect</x:v>
+      </x:c>
+      <x:c r="G3" s="103" t="str">
+        <x:v>Reason</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>Monthly innovation draw</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>2% per eligible product</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>Beer / Corona Extra is selected in Year 2, Month 3</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>None yet</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
+        <x:v>None yet</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="str">
+        <x:v>Every product receives an independent innovation chance each month.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Create variant name</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
+        <x:v>Month + year + serial</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>Corona Extra_M03_Y02_0127</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>Variant becomes a separate product row</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
+        <x:v>Variant becomes a separate product row</x:v>
+      </x:c>
+      <x:c r="G5" s="11" t="str">
+        <x:v>Keeps parent/child history easy to audit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Random launch price</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="str">
+        <x:v>85%–115% of parent current price</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>$18.99 parent → random price around that level</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>New price affects its own elastic demand</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>Nominal revenue uses launch price</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="str">
+        <x:v>Allows premium and discount variants.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>Transfer demand</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="str">
+        <x:v>10% of parent baseline spending</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
+        <x:v>10% moves from Corona Extra to its new variant</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>Total baseline household budget is preserved</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G7" s="11" t="str">
+        <x:v>New products should not manufacture consumer spending from nothing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>Transfer output</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="str">
+        <x:v>10% of parent output/inventory</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
+        <x:v>Parent output 1,000 → parent 900 + new variant 100</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
+        <x:v>Total physical capacity is initially preserved</x:v>
+      </x:c>
+      <x:c r="G8" s="11" t="str">
+        <x:v>Product variety alone should not create real GDP.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Elasticity</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="str">
+        <x:v>Parent ± random noise</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
+        <x:v>0.40 parent → e.g. 0.44 variant</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="str">
+        <x:v>Variant can respond differently to price</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G9" s="11" t="str">
+        <x:v>Related products are similar but not identical.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>Future evolution</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="str">
+        <x:v>Normal simulation rules</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>Demand, prices, production, entry/exit evolve after launch</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>Can gain or lose market share</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:v>Can expand or contract</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="str">
+        <x:v>The new product becomes a normal product after creation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="106" t="str">
+        <x:v>Note: with 2% monthly probability and new variants also eligible to innovate, the expected product count compounds over time. Starting from 477 products, 10 years can produce several thousand products. Set 'new_products_can_innovate' to 0 or use a monthly cap if you want slower variety growth.</x:v>
+      </x:c>
+      <x:c r="B12" s="106"/>
+      <x:c r="C12" s="106"/>
+      <x:c r="D12" s="106"/>
+      <x:c r="E12" s="106"/>
+      <x:c r="F12" s="106"/>
+      <x:c r="G12" s="106"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A12:G12"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1077,7 +1361,7 @@
       <x:c r="B21" s="11" t="str">
         <x:v>Entry: shortage weight</x:v>
       </x:c>
-      <x:c r="C21" s="80" t="n">
+      <x:c r="C21" s="75" t="n">
         <x:v>0.45</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
@@ -1097,7 +1381,7 @@
       <x:c r="B22" s="11" t="str">
         <x:v>Entry: demand growth weight</x:v>
       </x:c>
-      <x:c r="C22" s="80" t="n">
+      <x:c r="C22" s="75" t="n">
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="D22" s="11" t="str">
@@ -1117,7 +1401,7 @@
       <x:c r="B23" s="11" t="str">
         <x:v>Entry: profit margin weight</x:v>
       </x:c>
-      <x:c r="C23" s="80" t="n">
+      <x:c r="C23" s="75" t="n">
         <x:v>0.25</x:v>
       </x:c>
       <x:c r="D23" s="11" t="str">
@@ -1137,7 +1421,7 @@
       <x:c r="B24" s="11" t="str">
         <x:v>Exit: surplus weight</x:v>
       </x:c>
-      <x:c r="C24" s="80" t="n">
+      <x:c r="C24" s="75" t="n">
         <x:v>0.4</x:v>
       </x:c>
       <x:c r="D24" s="11" t="str">
@@ -1157,7 +1441,7 @@
       <x:c r="B25" s="11" t="str">
         <x:v>Exit: demand decline weight</x:v>
       </x:c>
-      <x:c r="C25" s="80" t="n">
+      <x:c r="C25" s="75" t="n">
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="D25" s="11" t="str">
@@ -1177,7 +1461,7 @@
       <x:c r="B26" s="11" t="str">
         <x:v>Exit: loss weight</x:v>
       </x:c>
-      <x:c r="C26" s="80" t="n">
+      <x:c r="C26" s="75" t="n">
         <x:v>0.3</x:v>
       </x:c>
       <x:c r="D26" s="11" t="str">
@@ -1197,7 +1481,7 @@
       <x:c r="B27" s="11" t="str">
         <x:v>Max entrants / product / year</x:v>
       </x:c>
-      <x:c r="C27" s="81" t="n">
+      <x:c r="C27" s="62" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="D27" s="11" t="str">
@@ -1217,7 +1501,7 @@
       <x:c r="B28" s="11" t="str">
         <x:v>Max exits / product / year</x:v>
       </x:c>
-      <x:c r="C28" s="81" t="n">
+      <x:c r="C28" s="62" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="D28" s="11" t="str">
@@ -1257,7 +1541,7 @@
       <x:c r="B30" s="11" t="str">
         <x:v>Exit capacity share</x:v>
       </x:c>
-      <x:c r="C30" s="80" t="n">
+      <x:c r="C30" s="75" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D30" s="11" t="str">
@@ -1277,7 +1561,7 @@
       <x:c r="B31" s="11" t="str">
         <x:v>Minimum entry score</x:v>
       </x:c>
-      <x:c r="C31" s="80" t="n">
+      <x:c r="C31" s="75" t="n">
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="D31" s="11" t="str">
@@ -1297,7 +1581,7 @@
       <x:c r="B32" s="11" t="str">
         <x:v>Minimum exit score</x:v>
       </x:c>
-      <x:c r="C32" s="80" t="n">
+      <x:c r="C32" s="75" t="n">
         <x:v>0.15</x:v>
       </x:c>
       <x:c r="D32" s="11" t="str">
@@ -1308,6 +1592,186 @@
       </x:c>
       <x:c r="F32" s="11" t="str">
         <x:v>A weak market must reach this score before recession-driven exits are allocated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="11" t="str">
+        <x:v>product_innovation_chance</x:v>
+      </x:c>
+      <x:c r="B33" s="11" t="str">
+        <x:v>Monthly new-product chance</x:v>
+      </x:c>
+      <x:c r="C33" s="95" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="D33" s="11" t="str">
+        <x:v>% per product / month</x:v>
+      </x:c>
+      <x:c r="E33" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F33" s="11" t="str">
+        <x:v>Each eligible existing product independently has this monthly probability of spawning one new variant.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="11" t="str">
+        <x:v>innovation_demand_share</x:v>
+      </x:c>
+      <x:c r="B34" s="11" t="str">
+        <x:v>Demand transferred to new variant</x:v>
+      </x:c>
+      <x:c r="C34" s="95" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D34" s="11" t="str">
+        <x:v>% of parent baseline spending</x:v>
+      </x:c>
+      <x:c r="E34" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F34" s="11" t="str">
+        <x:v>The launch initially takes this share of the parent product's baseline demand instead of creating demand from nothing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="11" t="str">
+        <x:v>innovation_output_share</x:v>
+      </x:c>
+      <x:c r="B35" s="11" t="str">
+        <x:v>Production transferred to new variant</x:v>
+      </x:c>
+      <x:c r="C35" s="95" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D35" s="11" t="str">
+        <x:v>% of parent output</x:v>
+      </x:c>
+      <x:c r="E35" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F35" s="11" t="str">
+        <x:v>The launch initially receives this share of the parent's current production and inventory.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="11" t="str">
+        <x:v>innovation_price_min_multiplier</x:v>
+      </x:c>
+      <x:c r="B36" s="11" t="str">
+        <x:v>Minimum launch-price multiplier</x:v>
+      </x:c>
+      <x:c r="C36" s="96" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="D36" s="11" t="str">
+        <x:v>x parent current price</x:v>
+      </x:c>
+      <x:c r="E36" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F36" s="11" t="str">
+        <x:v>Lower bound for the new product's random launch price.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="11" t="str">
+        <x:v>innovation_price_max_multiplier</x:v>
+      </x:c>
+      <x:c r="B37" s="11" t="str">
+        <x:v>Maximum launch-price multiplier</x:v>
+      </x:c>
+      <x:c r="C37" s="96" t="n">
+        <x:v>1.15</x:v>
+      </x:c>
+      <x:c r="D37" s="11" t="str">
+        <x:v>x parent current price</x:v>
+      </x:c>
+      <x:c r="E37" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F37" s="11" t="str">
+        <x:v>Upper bound for the new product's random launch price.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="11" t="str">
+        <x:v>innovation_elasticity_noise</x:v>
+      </x:c>
+      <x:c r="B38" s="11" t="str">
+        <x:v>Elasticity variation</x:v>
+      </x:c>
+      <x:c r="C38" s="96" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="D38" s="11" t="str">
+        <x:v>std. dev.</x:v>
+      </x:c>
+      <x:c r="E38" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F38" s="11" t="str">
+        <x:v>New variant inherits parent elasticity plus random normal variation; final elasticity is clipped to 0–1.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="11" t="str">
+        <x:v>innovation_initial_firms</x:v>
+      </x:c>
+      <x:c r="B39" s="11" t="str">
+        <x:v>Initial firms for new product</x:v>
+      </x:c>
+      <x:c r="C39" s="97" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D39" s="11" t="str">
+        <x:v>firms</x:v>
+      </x:c>
+      <x:c r="E39" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F39" s="11" t="str">
+        <x:v>A newly launched variant starts with this many producers; default 1 means a temporary monopoly.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="11" t="str">
+        <x:v>max_new_products_per_month</x:v>
+      </x:c>
+      <x:c r="B40" s="11" t="str">
+        <x:v>Maximum new products / month</x:v>
+      </x:c>
+      <x:c r="C40" s="97" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="11" t="str">
+        <x:v>products</x:v>
+      </x:c>
+      <x:c r="E40" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F40" s="11" t="str">
+        <x:v>0 means no cap. A positive value limits monthly launches after the probability draw.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="11" t="str">
+        <x:v>new_products_can_innovate</x:v>
+      </x:c>
+      <x:c r="B41" s="11" t="str">
+        <x:v>New variants can spawn variants</x:v>
+      </x:c>
+      <x:c r="C41" s="97" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D41" s="11" t="str">
+        <x:v>0/1</x:v>
+      </x:c>
+      <x:c r="E41" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F41" s="11" t="str">
+        <x:v>1 means all products, including previously created variants, can innovate in later months.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add Phase 2 employment wages and household income
</commit_message>
<xml_diff>
--- a/data/Simulation_Settings.xlsx
+++ b/data/Simulation_Settings.xlsx
@@ -2,16 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf8924302aa5743f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="R253b06d823cd4fa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="Rd4cff3d5aa8f4835"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="R62d1a7f3576d4730"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="R29d7d3d2066d4907"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="R883ffc0e2b6245e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption_Baskets" sheetId="7" r:id="R15f7eba23f944892"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase1_Model" sheetId="8" r:id="R4d4c5d067ddb4f22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firm_Entry_Exit" sheetId="9" r:id="R763e1afaebae4cdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Innovation" sheetId="10" r:id="Rbae576de4ac14fcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R33091b61ddd44ee0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="R7759989702f84ed2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="R21cc2f4831ff4187"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="Ra2957c2aab9044f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="Rd0b2f0857236491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="R3aa07d7e04fd4f83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption_Baskets" sheetId="7" r:id="R199a616bf56649b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase1_Model" sheetId="8" r:id="R3dad588681044ec1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firm_Entry_Exit" sheetId="9" r:id="Rece80f3138444374"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Innovation" sheetId="10" r:id="Recf497db08234125"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employment_Settings" sheetId="11" r:id="Rd6252a49e32841ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase2_Model" sheetId="12" r:id="R7a10a88c42f5441f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -58,7 +60,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -135,6 +137,26 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -143,7 +165,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="107">
+  <x:cellXfs count="126">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -323,6 +345,39 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -964,6 +1019,445 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="121" t="str">
+        <x:v>Phase 2 — Employment, Wages, and Household Income by Class</x:v>
+      </x:c>
+      <x:c r="B1" s="121"/>
+      <x:c r="C1" s="121"/>
+      <x:c r="D1" s="121"/>
+      <x:c r="E1" s="121"/>
+      <x:c r="F1" s="121"/>
+      <x:c r="G1" s="121"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11" t="str">
+        <x:v>Wage multipliers shape labor income across classes; capital-income weights shape ownership/business income. The engine normalizes both sets of weights each month, so aggregate labor and capital income reconcile exactly.</x:v>
+      </x:c>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+      <x:c r="G2" s="11"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="11"/>
+      <x:c r="C3" s="11"/>
+      <x:c r="D3" s="11"/>
+      <x:c r="E3" s="11"/>
+      <x:c r="F3" s="11"/>
+      <x:c r="G3" s="11"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="120" t="str">
+        <x:v>Order</x:v>
+      </x:c>
+      <x:c r="B4" s="120" t="str">
+        <x:v>Class</x:v>
+      </x:c>
+      <x:c r="C4" s="120" t="str">
+        <x:v>Wage Multiplier</x:v>
+      </x:c>
+      <x:c r="D4" s="120" t="str">
+        <x:v>Capital Income Weight</x:v>
+      </x:c>
+      <x:c r="E4" s="120" t="str">
+        <x:v>Labor-Force Participation Multiplier</x:v>
+      </x:c>
+      <x:c r="F4" s="120" t="str">
+        <x:v>Editable?</x:v>
+      </x:c>
+      <x:c r="G4" s="120" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="C5" s="114" t="n">
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="D5" s="114" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="E5" s="114" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G5" s="11" t="str">
+        <x:v>Lower average wage and relatively little capital income.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Middle</x:v>
+      </x:c>
+      <x:c r="C6" s="114" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" s="114" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="E6" s="114" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="str">
+        <x:v>Reference wage group.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="C7" s="114" t="n">
+        <x:v>1.55</x:v>
+      </x:c>
+      <x:c r="D7" s="114" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E7" s="114" t="n">
+        <x:v>1.05</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G7" s="11" t="str">
+        <x:v>Higher wages and more capital/business income.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>Top 1%</x:v>
+      </x:c>
+      <x:c r="C8" s="114" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="D8" s="114" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E8" s="114" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G8" s="11" t="str">
+        <x:v>High wage income plus concentrated capital income.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Top 0.1%</x:v>
+      </x:c>
+      <x:c r="C9" s="114" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D9" s="114" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E9" s="114" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="G9" s="11" t="str">
+        <x:v>Very concentrated capital/business income.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A2:G2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="54" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="121" t="str">
+        <x:v>Phase 2 — Labor Market and Household Income Flow</x:v>
+      </x:c>
+      <x:c r="B1" s="121"/>
+      <x:c r="C1" s="121"/>
+      <x:c r="D1" s="121"/>
+      <x:c r="E1" s="121"/>
+      <x:c r="F1" s="121"/>
+      <x:c r="G1" s="121"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11"/>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+      <x:c r="G2" s="11"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="120" t="str">
+        <x:v>Step</x:v>
+      </x:c>
+      <x:c r="B3" s="120" t="str">
+        <x:v>Mechanism</x:v>
+      </x:c>
+      <x:c r="C3" s="120" t="str">
+        <x:v>Driver</x:v>
+      </x:c>
+      <x:c r="D3" s="120" t="str">
+        <x:v>Economic effect</x:v>
+      </x:c>
+      <x:c r="E3" s="120" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="F3" s="120" t="str">
+        <x:v>Frequency</x:v>
+      </x:c>
+      <x:c r="G3" s="120" t="str">
+        <x:v>Phase-2 simplification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>Labor force</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>Households × participation rate</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>Demographic growth expands labor supply.</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>Labor force</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="str">
+        <x:v>One household represents one worker unit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Desired employment</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
+        <x:v>Real production + real wage + productivity</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>More real output raises labor demand; productivity lowers labor required.</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>Labor demand</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="G5" s="11" t="str">
+        <x:v>Employment demand responds to output and real wages; the wage elasticity is configurable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Actual employment</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="str">
+        <x:v>min(labor demand, labor force)</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>Weak demand creates unemployment; labor scarcity can constrain production.</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>Employment + unemployment</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="str">
+        <x:v>Labor is allocated proportionally across household classes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>Wage formation</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="str">
+        <x:v>Inflation + labor-market tightness</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
+        <x:v>Tight labor markets raise wages; slack labor markets slow/reduce wage growth.</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>Average wage</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="G7" s="11" t="str">
+        <x:v>One economy-wide wage index, with class wage multipliers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>Labor income</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="str">
+        <x:v>Employment × wage</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
+        <x:v>Company production now creates household wage income.</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
+        <x:v>Labor income by class</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="G8" s="11" t="str">
+        <x:v>Class wage multipliers are normalized to the aggregate wage bill.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Capital income</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="str">
+        <x:v>GDP − labor income</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
+        <x:v>Remaining national income is distributed using class capital-income weights.</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="str">
+        <x:v>Capital income by class</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="G9" s="11" t="str">
+        <x:v>Provides accounting closure until investment/government sectors are added.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>Household budget</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="str">
+        <x:v>Labor + capital + transfers − taxes</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>Consumption demand now responds to actual household income.</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>Consumption budget by class</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:v>Monthly</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="str">
+        <x:v>Savings remains zero for now.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
+        <x:v>Feedback loop</x:v>
+      </x:c>
+      <x:c r="C11" s="11" t="str">
+        <x:v>Income → demand → production → employment → income</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="str">
+        <x:v>Creates the first complete household/company circular-flow feedback.</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="str">
+        <x:v>GDP, wages, unemployment, class incomes</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="str">
+        <x:v>Every month</x:v>
+      </x:c>
+      <x:c r="G11" s="11" t="str">
+        <x:v>Government and financial markets remain future phases.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1601,7 +2095,7 @@
       <x:c r="B33" s="11" t="str">
         <x:v>Monthly new-product chance</x:v>
       </x:c>
-      <x:c r="C33" s="95" t="n">
+      <x:c r="C33" s="61" t="n">
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="D33" s="11" t="str">
@@ -1621,7 +2115,7 @@
       <x:c r="B34" s="11" t="str">
         <x:v>Demand transferred to new variant</x:v>
       </x:c>
-      <x:c r="C34" s="95" t="n">
+      <x:c r="C34" s="61" t="n">
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="D34" s="11" t="str">
@@ -1641,7 +2135,7 @@
       <x:c r="B35" s="11" t="str">
         <x:v>Production transferred to new variant</x:v>
       </x:c>
-      <x:c r="C35" s="95" t="n">
+      <x:c r="C35" s="61" t="n">
         <x:v>0.1</x:v>
       </x:c>
       <x:c r="D35" s="11" t="str">
@@ -1661,7 +2155,7 @@
       <x:c r="B36" s="11" t="str">
         <x:v>Minimum launch-price multiplier</x:v>
       </x:c>
-      <x:c r="C36" s="96" t="n">
+      <x:c r="C36" s="75" t="n">
         <x:v>0.85</x:v>
       </x:c>
       <x:c r="D36" s="11" t="str">
@@ -1681,7 +2175,7 @@
       <x:c r="B37" s="11" t="str">
         <x:v>Maximum launch-price multiplier</x:v>
       </x:c>
-      <x:c r="C37" s="96" t="n">
+      <x:c r="C37" s="75" t="n">
         <x:v>1.15</x:v>
       </x:c>
       <x:c r="D37" s="11" t="str">
@@ -1701,7 +2195,7 @@
       <x:c r="B38" s="11" t="str">
         <x:v>Elasticity variation</x:v>
       </x:c>
-      <x:c r="C38" s="96" t="n">
+      <x:c r="C38" s="75" t="n">
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="D38" s="11" t="str">
@@ -1721,7 +2215,7 @@
       <x:c r="B39" s="11" t="str">
         <x:v>Initial firms for new product</x:v>
       </x:c>
-      <x:c r="C39" s="97" t="n">
+      <x:c r="C39" s="62" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D39" s="11" t="str">
@@ -1741,7 +2235,7 @@
       <x:c r="B40" s="11" t="str">
         <x:v>Maximum new products / month</x:v>
       </x:c>
-      <x:c r="C40" s="97" t="n">
+      <x:c r="C40" s="62" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D40" s="11" t="str">
@@ -1761,7 +2255,7 @@
       <x:c r="B41" s="11" t="str">
         <x:v>New variants can spawn variants</x:v>
       </x:c>
-      <x:c r="C41" s="97" t="n">
+      <x:c r="C41" s="62" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D41" s="11" t="str">
@@ -1772,6 +2266,206 @@
       </x:c>
       <x:c r="F41" s="11" t="str">
         <x:v>1 means all products, including previously created variants, can innovate in later months.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="11" t="str">
+        <x:v>labor_force_participation</x:v>
+      </x:c>
+      <x:c r="B42" s="11" t="str">
+        <x:v>Labor-force participation</x:v>
+      </x:c>
+      <x:c r="C42" s="61" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="D42" s="11" t="str">
+        <x:v>% households</x:v>
+      </x:c>
+      <x:c r="E42" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F42" s="11" t="str">
+        <x:v>Potential workers as a share of households. Phase 2 treats one household as one representative worker unit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="11" t="str">
+        <x:v>initial_unemployment_rate</x:v>
+      </x:c>
+      <x:c r="B43" s="11" t="str">
+        <x:v>Initial unemployment rate</x:v>
+      </x:c>
+      <x:c r="C43" s="61" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="D43" s="11" t="str">
+        <x:v>% labor force</x:v>
+      </x:c>
+      <x:c r="E43" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F43" s="11" t="str">
+        <x:v>Used to calibrate Period-0 employment and the starting average wage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="11" t="str">
+        <x:v>labor_income_share_p0</x:v>
+      </x:c>
+      <x:c r="B44" s="11" t="str">
+        <x:v>Period-0 labor income share</x:v>
+      </x:c>
+      <x:c r="C44" s="61" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="D44" s="11" t="str">
+        <x:v>% GDP</x:v>
+      </x:c>
+      <x:c r="E44" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F44" s="11" t="str">
+        <x:v>Calibrates the starting wage bill. Remaining national income is allocated as capital income.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="11" t="str">
+        <x:v>labor_output_elasticity</x:v>
+      </x:c>
+      <x:c r="B45" s="11" t="str">
+        <x:v>Employment/output elasticity</x:v>
+      </x:c>
+      <x:c r="C45" s="75" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="D45" s="11" t="str">
+        <x:v>elasticity</x:v>
+      </x:c>
+      <x:c r="E45" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F45" s="11" t="str">
+        <x:v>How strongly desired employment changes when real production changes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="11" t="str">
+        <x:v>annual_labor_productivity_growth</x:v>
+      </x:c>
+      <x:c r="B46" s="11" t="str">
+        <x:v>Labor productivity growth</x:v>
+      </x:c>
+      <x:c r="C46" s="75" t="n">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="D46" s="11" t="str">
+        <x:v>% annual</x:v>
+      </x:c>
+      <x:c r="E46" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F46" s="11" t="str">
+        <x:v>Higher productivity lowers workers required for a given real output level.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="11" t="str">
+        <x:v>wage_adjustment_speed</x:v>
+      </x:c>
+      <x:c r="B47" s="11" t="str">
+        <x:v>Wage adjustment speed</x:v>
+      </x:c>
+      <x:c r="C47" s="75" t="n">
+        <x:v>0.08</x:v>
+      </x:c>
+      <x:c r="D47" s="11" t="str">
+        <x:v>coefficient</x:v>
+      </x:c>
+      <x:c r="E47" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F47" s="11" t="str">
+        <x:v>Monthly wage response to labor-market tightness.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="11" t="str">
+        <x:v>wage_inflation_pass_through</x:v>
+      </x:c>
+      <x:c r="B48" s="11" t="str">
+        <x:v>Inflation pass-through to wages</x:v>
+      </x:c>
+      <x:c r="C48" s="75" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D48" s="11" t="str">
+        <x:v>coefficient</x:v>
+      </x:c>
+      <x:c r="E48" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F48" s="11" t="str">
+        <x:v>Share of prior monthly inflation passed into the next month's wage change.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="11" t="str">
+        <x:v>max_monthly_wage_change</x:v>
+      </x:c>
+      <x:c r="B49" s="11" t="str">
+        <x:v>Maximum monthly wage change</x:v>
+      </x:c>
+      <x:c r="C49" s="61" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="D49" s="11" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="E49" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F49" s="11" t="str">
+        <x:v>Caps average wage increases/decreases in one month.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="11" t="str">
+        <x:v>unemployment_transfer_rate</x:v>
+      </x:c>
+      <x:c r="B50" s="11" t="str">
+        <x:v>Unemployment transfer rate</x:v>
+      </x:c>
+      <x:c r="C50" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D50" s="11" t="str">
+        <x:v>% average wage</x:v>
+      </x:c>
+      <x:c r="E50" s="11" t="str">
+        <x:v>Stored</x:v>
+      </x:c>
+      <x:c r="F50" s="11" t="str">
+        <x:v>Optional transfer per unemployed worker unit. Default 0 until the government sector is modeled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="11" t="str">
+        <x:v>labor_wage_demand_elasticity</x:v>
+      </x:c>
+      <x:c r="B51" s="11" t="str">
+        <x:v>Labor demand / real-wage elasticity</x:v>
+      </x:c>
+      <x:c r="C51" s="125" t="n">
+        <x:v>0.35</x:v>
+      </x:c>
+      <x:c r="D51" s="11" t="str">
+        <x:v>elasticity</x:v>
+      </x:c>
+      <x:c r="E51" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F51" s="11" t="str">
+        <x:v>Lower real wages increase desired employment and higher real wages reduce it; stabilizes the labor market.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add Phase 3 government taxes transfers and public debt
</commit_message>
<xml_diff>
--- a/data/Simulation_Settings.xlsx
+++ b/data/Simulation_Settings.xlsx
@@ -2,18 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R33091b61ddd44ee0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="R7759989702f84ed2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="R21cc2f4831ff4187"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="Ra2957c2aab9044f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="Rd0b2f0857236491b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="R3aa07d7e04fd4f83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption_Baskets" sheetId="7" r:id="R199a616bf56649b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase1_Model" sheetId="8" r:id="R3dad588681044ec1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firm_Entry_Exit" sheetId="9" r:id="Rece80f3138444374"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Innovation" sheetId="10" r:id="Recf497db08234125"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employment_Settings" sheetId="11" r:id="Rd6252a49e32841ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase2_Model" sheetId="12" r:id="R7a10a88c42f5441f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rb19574ca78c64267"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="General_Settings" sheetId="2" r:id="R78c3db833af04f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Household_Classes" sheetId="3" r:id="R7c6ea50ff1da41d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company_Settings" sheetId="4" r:id="R1376557c43174b43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quantity_Limits" sheetId="5" r:id="R0bdc65737f474cd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Summary" sheetId="6" r:id="R64cf093854b64cab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumption_Baskets" sheetId="7" r:id="R4241779dd33b4e03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase1_Model" sheetId="8" r:id="Ree2277c4e4994692"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firm_Entry_Exit" sheetId="9" r:id="Rd586d8f11ac442b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product_Innovation" sheetId="10" r:id="Rc9b925b822d34d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employment_Settings" sheetId="11" r:id="R08e2b3bf36424545"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase2_Model" sheetId="12" r:id="R94aa9478c9054b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Government_Transfers" sheetId="13" r:id="R44eccd62e7f34ca7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Government_Demand" sheetId="14" r:id="Rac78bc97b94e4fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase3_Model" sheetId="15" r:id="R0b7b5d16341f4e60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -60,7 +63,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="20">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -157,6 +160,21 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -165,7 +183,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="126">
+  <x:cellXfs count="142">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -378,6 +396,36 @@
     <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="205" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="205" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1458,6 +1506,689 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="55" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="139" t="str">
+        <x:v>Phase 3 — Government Transfer Distribution</x:v>
+      </x:c>
+      <x:c r="B1" s="139"/>
+      <x:c r="C1" s="139"/>
+      <x:c r="D1" s="139"/>
+      <x:c r="E1" s="139"/>
+      <x:c r="F1" s="139"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11" t="str">
+        <x:v>Weights distribute the general transfer pool across household classes. They are relative weights, not percentages.</x:v>
+      </x:c>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="11"/>
+      <x:c r="C3" s="11"/>
+      <x:c r="D3" s="11"/>
+      <x:c r="E3" s="11"/>
+      <x:c r="F3" s="11"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="137" t="str">
+        <x:v>Order</x:v>
+      </x:c>
+      <x:c r="B4" s="137" t="str">
+        <x:v>Class</x:v>
+      </x:c>
+      <x:c r="C4" s="137" t="str">
+        <x:v>Transfer Weight</x:v>
+      </x:c>
+      <x:c r="D4" s="137" t="str">
+        <x:v>Taxable?</x:v>
+      </x:c>
+      <x:c r="E4" s="137" t="str">
+        <x:v>Editable?</x:v>
+      </x:c>
+      <x:c r="F4" s="137" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="C5" s="140" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
+        <x:v>Highest relative eligibility for general transfers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Middle</x:v>
+      </x:c>
+      <x:c r="C6" s="140" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>Moderate transfer weight.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="C7" s="140" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="str">
+        <x:v>Small transfer weight.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>Top 1%</x:v>
+      </x:c>
+      <x:c r="C8" s="140" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
+        <x:v>No default general transfer.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Top 0.1%</x:v>
+      </x:c>
+      <x:c r="C9" s="140" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="str">
+        <x:v>No default general transfer.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="55" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="139" t="str">
+        <x:v>Phase 3 — Government Purchases by COICOP Division</x:v>
+      </x:c>
+      <x:c r="B1" s="139"/>
+      <x:c r="C1" s="139"/>
+      <x:c r="D1" s="139"/>
+      <x:c r="E1" s="139"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11" t="str">
+        <x:v>Weights tilt public purchases by COICOP division. Product allocation is proportional to current production value × the editable division priority weight.</x:v>
+      </x:c>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="11"/>
+      <x:c r="B3" s="11"/>
+      <x:c r="C3" s="11"/>
+      <x:c r="D3" s="11"/>
+      <x:c r="E3" s="11"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="137" t="str">
+        <x:v>Division</x:v>
+      </x:c>
+      <x:c r="B4" s="137" t="str">
+        <x:v>COICOP Division</x:v>
+      </x:c>
+      <x:c r="C4" s="137" t="str">
+        <x:v>Government Weight</x:v>
+      </x:c>
+      <x:c r="D4" s="137" t="str">
+        <x:v>Editable?</x:v>
+      </x:c>
+      <x:c r="E4" s="137" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="str">
+        <x:v>01</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Food &amp; non-alcoholic beverages</x:v>
+      </x:c>
+      <x:c r="C5" s="140" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>Public institutions / food programs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="str">
+        <x:v>02</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Alcohol &amp; tobacco</x:v>
+      </x:c>
+      <x:c r="C6" s="140" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>No default government purchases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="str">
+        <x:v>03</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>Clothing &amp; footwear</x:v>
+      </x:c>
+      <x:c r="C7" s="140" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>Uniforms and public-service supplies.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="str">
+        <x:v>04</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>Housing &amp; utilities</x:v>
+      </x:c>
+      <x:c r="C8" s="140" t="n">
+        <x:v>1.2</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
+        <x:v>Public buildings, utilities and housing services.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="str">
+        <x:v>05</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Furnishings &amp; maintenance</x:v>
+      </x:c>
+      <x:c r="C9" s="140" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="str">
+        <x:v>Maintenance and operating supplies.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="str">
+        <x:v>06</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>Health</x:v>
+      </x:c>
+      <x:c r="C10" s="140" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>High public health/services weight.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="11" t="str">
+        <x:v>07</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
+        <x:v>Transport</x:v>
+      </x:c>
+      <x:c r="C11" s="140" t="n">
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="str">
+        <x:v>Transport/infrastructure-related purchases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="11" t="str">
+        <x:v>08</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="str">
+        <x:v>Communication</x:v>
+      </x:c>
+      <x:c r="C12" s="140" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E12" s="11" t="str">
+        <x:v>Government communications/services.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="11" t="str">
+        <x:v>09</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>Recreation</x:v>
+      </x:c>
+      <x:c r="C13" s="140" t="n">
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="D13" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="str">
+        <x:v>Parks/recreation/cultural spending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="11" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="11" t="str">
+        <x:v>Education</x:v>
+      </x:c>
+      <x:c r="C14" s="140" t="n">
+        <x:v>2.5</x:v>
+      </x:c>
+      <x:c r="D14" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="str">
+        <x:v>High public education weight.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="11" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B15" s="11" t="str">
+        <x:v>Restaurants &amp; hotels</x:v>
+      </x:c>
+      <x:c r="C15" s="140" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E15" s="11" t="str">
+        <x:v>Limited travel/hospitality demand.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="11" t="str">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="str">
+        <x:v>Financial, insurance &amp; services</x:v>
+      </x:c>
+      <x:c r="C16" s="140" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="E16" s="11" t="str">
+        <x:v>Professional, legal and financial services.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="139" t="str">
+        <x:v>Phase 3 — Government, Taxes, Transfers, Spending and Debt</x:v>
+      </x:c>
+      <x:c r="B1" s="139"/>
+      <x:c r="C1" s="139"/>
+      <x:c r="D1" s="139"/>
+      <x:c r="E1" s="139"/>
+      <x:c r="F1" s="139"/>
+      <x:c r="G1" s="139"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="11"/>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+      <x:c r="G2" s="11"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="137" t="str">
+        <x:v>Step</x:v>
+      </x:c>
+      <x:c r="B3" s="137" t="str">
+        <x:v>Government flow</x:v>
+      </x:c>
+      <x:c r="C3" s="137" t="str">
+        <x:v>Source / rule</x:v>
+      </x:c>
+      <x:c r="D3" s="137" t="str">
+        <x:v>Economic effect</x:v>
+      </x:c>
+      <x:c r="E3" s="137" t="str">
+        <x:v>Monthly output</x:v>
+      </x:c>
+      <x:c r="F3" s="137" t="str">
+        <x:v>Default</x:v>
+      </x:c>
+      <x:c r="G3" s="137" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>Household income tax</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>20% of gross household income</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>Reduces disposable household consumption; creates government revenue.</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>Household_Tax_Revenue</x:v>
+      </x:c>
+      <x:c r="F4" s="11" t="str">
+        <x:v>20%</x:v>
+      </x:c>
+      <x:c r="G4" s="11" t="str">
+        <x:v>Editable in General_Settings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>Corporate profit tax</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
+        <x:v>20% of gross business/capital income</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>Moves part of company profit to government revenue.</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>Corporate_Tax_Revenue</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
+        <x:v>20%</x:v>
+      </x:c>
+      <x:c r="G5" s="11" t="str">
+        <x:v>Loss-making firms/products do not generate negative tax.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Unemployment benefits</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="str">
+        <x:v>30% of average wage × unemployed worker units</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>Supports household income during unemployment.</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>Unemployment_Benefits</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>30% wage</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="str">
+        <x:v>Paid by government and added to household transfers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>General transfers</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="str">
+        <x:v>20% of gross tax revenue distributed by class weights</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
+        <x:v>Redistributes income toward lower-income households.</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>General_Transfers</x:v>
+      </x:c>
+      <x:c r="F7" s="11" t="str">
+        <x:v>20% revenue</x:v>
+      </x:c>
+      <x:c r="G7" s="11" t="str">
+        <x:v>Class weights are editable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>Government purchases</x:v>
+      </x:c>
+      <x:c r="C8" s="11" t="str">
+        <x:v>80% of gross tax revenue allocated across products</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
+        <x:v>Creates direct government demand for goods/services.</x:v>
+      </x:c>
+      <x:c r="E8" s="11" t="str">
+        <x:v>Government_Purchases</x:v>
+      </x:c>
+      <x:c r="F8" s="11" t="str">
+        <x:v>80% revenue</x:v>
+      </x:c>
+      <x:c r="G8" s="11" t="str">
+        <x:v>Division weights are editable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>Debt interest</x:v>
+      </x:c>
+      <x:c r="C9" s="11" t="str">
+        <x:v>Annual rate / 12 × beginning public debt</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
+        <x:v>Raises government expenses when debt is outstanding.</x:v>
+      </x:c>
+      <x:c r="E9" s="11" t="str">
+        <x:v>Debt_Interest</x:v>
+      </x:c>
+      <x:c r="F9" s="11" t="str">
+        <x:v>3% annual</x:v>
+      </x:c>
+      <x:c r="G9" s="11" t="str">
+        <x:v>Editable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>Budget balance</x:v>
+      </x:c>
+      <x:c r="C10" s="11" t="str">
+        <x:v>Revenue − purchases − transfers − unemployment benefits − debt interest</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
+        <x:v>Surplus reduces debt; deficit increases debt.</x:v>
+      </x:c>
+      <x:c r="E10" s="11" t="str">
+        <x:v>Budget_Balance</x:v>
+      </x:c>
+      <x:c r="F10" s="11" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G10" s="11" t="str">
+        <x:v>Debt cannot fall below zero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
+        <x:v>Public debt</x:v>
+      </x:c>
+      <x:c r="C11" s="11" t="str">
+        <x:v>Prior debt − budget balance</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="str">
+        <x:v>Carries fiscal imbalances forward over time.</x:v>
+      </x:c>
+      <x:c r="E11" s="11" t="str">
+        <x:v>Public_Debt_End</x:v>
+      </x:c>
+      <x:c r="F11" s="11" t="str">
+        <x:v>$0 start</x:v>
+      </x:c>
+      <x:c r="G11" s="11" t="str">
+        <x:v>No bond-market feedback yet.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1533,19 +2264,19 @@
         <x:v>tax_rate</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>Taxes</x:v>
+        <x:v>Household income tax</x:v>
       </x:c>
       <x:c r="C5" s="61" t="n">
-        <x:v>0</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
-        <x:v>% of gross income</x:v>
+        <x:v>% gross household income</x:v>
       </x:c>
       <x:c r="E5" s="11" t="str">
         <x:v>Used</x:v>
       </x:c>
       <x:c r="F5" s="11" t="str">
-        <x:v>Flat household income-tax placeholder.</x:v>
+        <x:v>Flat household income tax. Phase 3 default = 20%. Revenue flows to the government sector.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2436,16 +3167,16 @@
         <x:v>Unemployment transfer rate</x:v>
       </x:c>
       <x:c r="C50" s="61" t="n">
-        <x:v>0</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="D50" s="11" t="str">
         <x:v>% average wage</x:v>
       </x:c>
       <x:c r="E50" s="11" t="str">
-        <x:v>Stored</x:v>
+        <x:v>Used</x:v>
       </x:c>
       <x:c r="F50" s="11" t="str">
-        <x:v>Optional transfer per unemployed worker unit. Default 0 until the government sector is modeled.</x:v>
+        <x:v>Government unemployment benefit per unemployed worker unit as a share of the current average wage.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -2455,7 +3186,7 @@
       <x:c r="B51" s="11" t="str">
         <x:v>Labor demand / real-wage elasticity</x:v>
       </x:c>
-      <x:c r="C51" s="125" t="n">
+      <x:c r="C51" s="75" t="n">
         <x:v>0.35</x:v>
       </x:c>
       <x:c r="D51" s="11" t="str">
@@ -2466,6 +3197,146 @@
       </x:c>
       <x:c r="F51" s="11" t="str">
         <x:v>Lower real wages increase desired employment and higher real wages reduce it; stabilizes the labor market.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="11" t="str">
+        <x:v>corporate_profit_tax_rate</x:v>
+      </x:c>
+      <x:c r="B52" s="11" t="str">
+        <x:v>Corporate profit tax</x:v>
+      </x:c>
+      <x:c r="C52" s="130" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D52" s="11" t="str">
+        <x:v>% positive profit</x:v>
+      </x:c>
+      <x:c r="E52" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F52" s="11" t="str">
+        <x:v>20% tax proxy on gross business/capital income before net capital income is distributed to households.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="11" t="str">
+        <x:v>government_consumption_share</x:v>
+      </x:c>
+      <x:c r="B53" s="11" t="str">
+        <x:v>Government purchases share</x:v>
+      </x:c>
+      <x:c r="C53" s="61" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="D53" s="11" t="str">
+        <x:v>% gross tax revenue</x:v>
+      </x:c>
+      <x:c r="E53" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F53" s="11" t="str">
+        <x:v>Default 80% of gross tax revenue is recycled through direct government purchases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="11" t="str">
+        <x:v>general_transfer_share</x:v>
+      </x:c>
+      <x:c r="B54" s="11" t="str">
+        <x:v>General transfer pool</x:v>
+      </x:c>
+      <x:c r="C54" s="61" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="D54" s="11" t="str">
+        <x:v>% gross tax revenue</x:v>
+      </x:c>
+      <x:c r="E54" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F54" s="11" t="str">
+        <x:v>Default 20% of gross tax revenue is recycled as household transfers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="11" t="str">
+        <x:v>government_reserve_share</x:v>
+      </x:c>
+      <x:c r="B55" s="11" t="str">
+        <x:v>Government reserve share</x:v>
+      </x:c>
+      <x:c r="C55" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D55" s="11" t="str">
+        <x:v>% gross tax revenue</x:v>
+      </x:c>
+      <x:c r="E55" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F55" s="11" t="str">
+        <x:v>Default 0%. Unemployment benefits and debt interest can therefore create a fiscal deficit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="11" t="str">
+        <x:v>initial_public_debt</x:v>
+      </x:c>
+      <x:c r="B56" s="11" t="str">
+        <x:v>Initial public debt</x:v>
+      </x:c>
+      <x:c r="C56" s="131" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D56" s="11" t="str">
+        <x:v>$</x:v>
+      </x:c>
+      <x:c r="E56" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F56" s="11" t="str">
+        <x:v>Starting nominal public debt. Monthly deficits increase debt; surpluses reduce it but not below zero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="11" t="str">
+        <x:v>debt_interest_rate</x:v>
+      </x:c>
+      <x:c r="B57" s="11" t="str">
+        <x:v>Public debt interest rate</x:v>
+      </x:c>
+      <x:c r="C57" s="130" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="D57" s="11" t="str">
+        <x:v>% annual</x:v>
+      </x:c>
+      <x:c r="E57" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F57" s="11" t="str">
+        <x:v>Annual interest charged on beginning public debt; interest is a government expense.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="11" t="str">
+        <x:v>max_government_demand_growth</x:v>
+      </x:c>
+      <x:c r="B58" s="11" t="str">
+        <x:v>Max monthly government-demand change</x:v>
+      </x:c>
+      <x:c r="C58" s="130" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D58" s="11" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="E58" s="11" t="str">
+        <x:v>Used</x:v>
+      </x:c>
+      <x:c r="F58" s="11" t="str">
+        <x:v>Caps changes in government-purchase budget caused by volatile tax revenue.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>